<commit_message>
Updated figures and dataframes
</commit_message>
<xml_diff>
--- a/data/2027 Country names and groupings.xlsx
+++ b/data/2027 Country names and groupings.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hedikatrekr/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F98EBD4-2E02-C046-98E6-2CBFD765D785}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{349357A0-CC59-1C4E-BDE4-ADFE0FD89AE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19720" yWindow="500" windowWidth="42080" windowHeight="25120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="European country names - ISO3 c" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,9 @@
         <t xml:space="preserve">[Trådad kommentar]
 I din version av Excel kan du läsa den här trådade kommentaren, men eventuella ändringar i den tas bort om filen öppnas i en senare version av Excel. Läs mer: https://go.microsoft.com/fwlink/?linkid=870924
 Kommentar:
-    EEA+UK=main results to be reported in the main text in the 2027 report. </t>
+    EEA+UK=main results to be reported in the main text in the 2027 report. 
+Svar:
+    For the subregions in the report please include UK to Northern Europe! In the data sheet, please provide the Europe estimates 1. EEA+  UK and 2. Only EEA (NO UK) and same for the subregions. </t>
       </text>
     </comment>
     <comment ref="G2" authorId="1" shapeId="0" xr:uid="{C5D1D998-4A6C-294A-92A7-B42BE925523D}">
@@ -702,7 +704,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -732,12 +734,6 @@
       <sz val="8"/>
       <color theme="1"/>
       <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Tahoma"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -986,6 +982,9 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -996,9 +995,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1224,6 +1220,9 @@
   <threadedComment ref="F2" dT="2025-11-28T08:50:26.83" personId="{EAFEAAD6-1398-7B45-B716-56CFC52763E8}" id="{5EB1477D-8865-AF47-ADC2-06529D902E1B}">
     <text xml:space="preserve">EEA+UK=main results to be reported in the main text in the 2027 report. </text>
   </threadedComment>
+  <threadedComment ref="F2" dT="2026-04-08T08:33:33.45" personId="{EAFEAAD6-1398-7B45-B716-56CFC52763E8}" id="{FC4295C1-75B2-6D4C-84EF-8602ECB4605B}" parentId="{5EB1477D-8865-AF47-ADC2-06529D902E1B}">
+    <text xml:space="preserve">For the subregions in the report please include UK to Northern Europe! In the data sheet, please provide the Europe estimates 1. EEA+  UK and 2. Only EEA (NO UK) and same for the subregions. </text>
+  </threadedComment>
   <threadedComment ref="G2" dT="2025-11-28T08:49:54.51" personId="{EAFEAAD6-1398-7B45-B716-56CFC52763E8}" id="{C5D1D998-4A6C-294A-92A7-B42BE925523D}">
     <text xml:space="preserve">If your indicator covers the WHO-53+Kosova and LIchtenshtein you can provide country level data with your data submission. </text>
   </threadedComment>
@@ -1253,30 +1252,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:53" s="1" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="25" t="s">
         <v>205</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
-      <c r="G1" s="25"/>
-      <c r="H1" s="25"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
+      <c r="G1" s="26"/>
+      <c r="H1" s="26"/>
       <c r="I1" s="21"/>
-      <c r="J1" s="24" t="s">
+      <c r="J1" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="K1" s="26"/>
-      <c r="L1" s="22" t="s">
+      <c r="K1" s="27"/>
+      <c r="L1" s="23" t="s">
         <v>1</v>
       </c>
-      <c r="M1" s="23"/>
-      <c r="N1" s="23"/>
-      <c r="O1" s="23"/>
-      <c r="P1" s="23"/>
-      <c r="Q1" s="23"/>
-      <c r="R1" s="23"/>
+      <c r="M1" s="24"/>
+      <c r="N1" s="24"/>
+      <c r="O1" s="24"/>
+      <c r="P1" s="24"/>
+      <c r="Q1" s="24"/>
+      <c r="R1" s="24"/>
     </row>
     <row r="2" spans="1:53" s="9" customFormat="1" ht="32" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="7" t="s">
@@ -1294,7 +1293,7 @@
       <c r="E2" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="F2" s="27" t="s">
+      <c r="F2" s="22" t="s">
         <v>206</v>
       </c>
       <c r="G2" s="7" t="s">
@@ -3351,8 +3350,242 @@
 </worksheet>
 </file>
 
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100BE999D9A6EB5694A9E61F56E0C65FA6E" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="7e3fa9533e1523351dc1a8c45d523838">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d2f08301-3572-41d6-bf1e-19bd96c47c4f" xmlns:ns3="4c3d6b82-f9af-440b-a18a-3e1dc74d2270" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="07f2a39ac6620e5ae12889bba8cde6ca" ns2:_="" ns3:_="">
+    <xsd:import namespace="d2f08301-3572-41d6-bf1e-19bd96c47c4f"/>
+    <xsd:import namespace="4c3d6b82-f9af-440b-a18a-3e1dc74d2270"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="d2f08301-3572-41d6-bf1e-19bd96c47c4f" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="11" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="1103e67f-0598-4a90-8a4a-cec34b03bfa0" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="13" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="14" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="15" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="16" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="18" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="19" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="4c3d6b82-f9af-440b-a18a-3e1dc74d2270" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="12" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{f05aecd8-fc53-422d-90b0-cfbb054cca51}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="4c3d6b82-f9af-440b-a18a-3e1dc74d2270">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="4c3d6b82-f9af-440b-a18a-3e1dc74d2270" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d2f08301-3572-41d6-bf1e-19bd96c47c4f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{217E3769-A85D-42FE-BEF4-90E081CDBB1E}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7E248C7E-E841-4BCC-B13D-4A075C2C2650}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A607E69A-05DF-4A45-9820-3331242C8597}"/>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
-  <clbl:label id="{f13b610e-d3b5-490f-b165-988100e8232a}" enabled="1" method="Standard" siteId="{5a4ba6f9-f531-4f32-9467-398f19e69de4}" contentBits="1" removed="0"/>
+  <clbl:label id="{912a5d77-fb98-4eee-af32-1334d8f04a53}" enabled="0" method="" siteId="{912a5d77-fb98-4eee-af32-1334d8f04a53}" removed="1"/>
+  <clbl:label id="{f13b610e-d3b5-490f-b165-988100e8232a}" enabled="1" method="Standard" siteId="{5a4ba6f9-f531-4f32-9467-398f19e69de4}" removed="0"/>
 </clbl:labelList>
 </file>
</xml_diff>